<commit_message>
fixed stats issue in CodeScene data
</commit_message>
<xml_diff>
--- a/design_issues/codescene/P10_POS.xlsx
+++ b/design_issues/codescene/P10_POS.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AI IDE Analysis\AI-IDEs-code-analysis\design_issues\codescene\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DIinAGP\DIinAGP\design_issues\codescene\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Issues" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="121">
   <si>
     <t>resource</t>
   </si>
@@ -329,12 +329,6 @@
   </si>
   <si>
     <t>/E:/AI IDE Analysis/AI-IDEs-code-analysis/projects/P10_POS/frontend/src/utils/indexedDB.ts</t>
-  </si>
-  <si>
-    <t>String Heavy Function Arguments</t>
-  </si>
-  <si>
-    <t>String Heavy Function Arguments ()</t>
   </si>
   <si>
     <t>/E:/AI IDE Analysis/AI-IDEs-code-analysis/projects/P10_POS/frontend/src/utils/syncManager.ts</t>
@@ -766,7 +760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E193"/>
+  <dimension ref="A1:E192"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="112" customWidth="1"/>
@@ -3620,16 +3614,16 @@
         <v>102</v>
       </c>
       <c r="B168" t="s">
-        <v>103</v>
+        <v>8</v>
       </c>
       <c r="C168" t="s">
-        <v>104</v>
+        <v>9</v>
       </c>
       <c r="D168">
-        <v>1</v>
+        <v>125</v>
       </c>
       <c r="E168">
-        <v>1</v>
+        <v>125</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.35">
@@ -3643,10 +3637,10 @@
         <v>9</v>
       </c>
       <c r="D169">
-        <v>125</v>
+        <v>172</v>
       </c>
       <c r="E169">
-        <v>125</v>
+        <v>172</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.35">
@@ -3660,10 +3654,10 @@
         <v>9</v>
       </c>
       <c r="D170">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="E170">
-        <v>172</v>
+        <v>187</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.35">
@@ -3677,10 +3671,10 @@
         <v>9</v>
       </c>
       <c r="D171">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="E171">
-        <v>187</v>
+        <v>202</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.35">
@@ -3694,10 +3688,10 @@
         <v>9</v>
       </c>
       <c r="D172">
-        <v>202</v>
+        <v>222</v>
       </c>
       <c r="E172">
-        <v>202</v>
+        <v>222</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.35">
@@ -3711,55 +3705,55 @@
         <v>9</v>
       </c>
       <c r="D173">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="E173">
-        <v>222</v>
+        <v>237</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B174" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C174" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D174">
-        <v>237</v>
+        <v>1</v>
       </c>
       <c r="E174">
-        <v>237</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B175" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="C175" t="s">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="D175">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="E175">
-        <v>1</v>
+        <v>99</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B176" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C176" t="s">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="D176">
         <v>99</v>
@@ -3770,13 +3764,13 @@
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B177" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C177" t="s">
-        <v>21</v>
+        <v>104</v>
       </c>
       <c r="D177">
         <v>99</v>
@@ -3787,13 +3781,13 @@
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
+        <v>103</v>
+      </c>
+      <c r="B178" t="s">
+        <v>23</v>
+      </c>
+      <c r="C178" t="s">
         <v>105</v>
-      </c>
-      <c r="B178" t="s">
-        <v>10</v>
-      </c>
-      <c r="C178" t="s">
-        <v>106</v>
       </c>
       <c r="D178">
         <v>99</v>
@@ -3804,75 +3798,75 @@
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B179" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C179" t="s">
-        <v>107</v>
+        <v>28</v>
       </c>
       <c r="D179">
-        <v>99</v>
+        <v>133</v>
       </c>
       <c r="E179">
-        <v>99</v>
+        <v>133</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B180" t="s">
         <v>10</v>
       </c>
       <c r="C180" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D180">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="E180">
-        <v>133</v>
+        <v>157</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B181" t="s">
         <v>10</v>
       </c>
       <c r="C181" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="D181">
-        <v>157</v>
+        <v>65</v>
       </c>
       <c r="E181">
-        <v>157</v>
+        <v>65</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B182" t="s">
         <v>10</v>
       </c>
       <c r="C182" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D182">
-        <v>65</v>
+        <v>159</v>
       </c>
       <c r="E182">
-        <v>65</v>
+        <v>159</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B183" t="s">
         <v>10</v>
@@ -3881,32 +3875,32 @@
         <v>38</v>
       </c>
       <c r="D183">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="E183">
-        <v>159</v>
+        <v>182</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B184" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C184" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="D184">
-        <v>182</v>
+        <v>119</v>
       </c>
       <c r="E184">
-        <v>182</v>
+        <v>119</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B185" t="s">
         <v>8</v>
@@ -3915,32 +3909,32 @@
         <v>9</v>
       </c>
       <c r="D185">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="E185">
-        <v>119</v>
+        <v>131</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B186" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C186" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D186">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="E186">
-        <v>131</v>
+        <v>116</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B187" t="s">
         <v>10</v>
@@ -3949,15 +3943,15 @@
         <v>11</v>
       </c>
       <c r="D187">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E187">
-        <v>116</v>
+        <v>111</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B188" t="s">
         <v>10</v>
@@ -3966,15 +3960,15 @@
         <v>11</v>
       </c>
       <c r="D188">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="E188">
-        <v>111</v>
+        <v>131</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B189" t="s">
         <v>10</v>
@@ -3983,77 +3977,60 @@
         <v>11</v>
       </c>
       <c r="D189">
-        <v>131</v>
+        <v>102</v>
       </c>
       <c r="E189">
-        <v>131</v>
+        <v>102</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B190" t="s">
         <v>10</v>
       </c>
       <c r="C190" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="D190">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="E190">
-        <v>102</v>
+        <v>141</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B191" t="s">
         <v>10</v>
       </c>
       <c r="C191" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="D191">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="E191">
-        <v>141</v>
+        <v>160</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B192" t="s">
         <v>10</v>
       </c>
       <c r="C192" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="D192">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="E192">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A193" t="s">
-        <v>118</v>
-      </c>
-      <c r="B193" t="s">
-        <v>10</v>
-      </c>
-      <c r="C193" t="s">
-        <v>38</v>
-      </c>
-      <c r="D193">
-        <v>139</v>
-      </c>
-      <c r="E193">
         <v>139</v>
       </c>
     </row>
@@ -4064,7 +4041,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:C16"/>
+  <dimension ref="A2:C15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="35.6328125" customWidth="1"/>
@@ -4073,13 +4050,13 @@
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>119</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -4090,7 +4067,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="2">
-        <f>COUNTIF(Issues!B2:B201,Stats!B3)</f>
+        <f>COUNTIF(Issues!B2:B200,Stats!B3)</f>
         <v>47</v>
       </c>
     </row>
@@ -4102,7 +4079,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="2">
-        <f>COUNTIF(Issues!B2:B202,Stats!B4)</f>
+        <f>COUNTIF(Issues!B2:B201,Stats!B4)</f>
         <v>13</v>
       </c>
     </row>
@@ -4114,7 +4091,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="2">
-        <f>COUNTIF(Issues!B2:B203,Stats!B5)</f>
+        <f>COUNTIF(Issues!B2:B202,Stats!B5)</f>
         <v>70</v>
       </c>
     </row>
@@ -4126,7 +4103,7 @@
         <v>23</v>
       </c>
       <c r="C6" s="2">
-        <f>COUNTIF(Issues!B2:B204,Stats!B6)</f>
+        <f>COUNTIF(Issues!B2:B203,Stats!B6)</f>
         <v>23</v>
       </c>
     </row>
@@ -4138,7 +4115,7 @@
         <v>25</v>
       </c>
       <c r="C7" s="2">
-        <f>COUNTIF(Issues!B2:B205,Stats!B7)</f>
+        <f>COUNTIF(Issues!B2:B204,Stats!B7)</f>
         <v>5</v>
       </c>
     </row>
@@ -4150,7 +4127,7 @@
         <v>50</v>
       </c>
       <c r="C8" s="2">
-        <f>COUNTIF(Issues!B2:B207,Stats!B8)</f>
+        <f>COUNTIF(Issues!B2:B206,Stats!B8)</f>
         <v>1</v>
       </c>
     </row>
@@ -4162,7 +4139,7 @@
         <v>18</v>
       </c>
       <c r="C9" s="2">
-        <f>COUNTIF(Issues!B2:B209,Stats!B9)</f>
+        <f>COUNTIF(Issues!B2:B208,Stats!B9)</f>
         <v>21</v>
       </c>
     </row>
@@ -4174,7 +4151,7 @@
         <v>88</v>
       </c>
       <c r="C10" s="2">
-        <f>COUNTIF(Issues!B2:B210,Stats!B10)</f>
+        <f>COUNTIF(Issues!B2:B209,Stats!B10)</f>
         <v>3</v>
       </c>
     </row>
@@ -4183,23 +4160,23 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2">
         <f>COUNTIF(Issues!B2:B211,Stats!B11)</f>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>10</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>20</v>
+      <c r="B12" t="s">
+        <v>13</v>
       </c>
       <c r="C12" s="2">
-        <f>COUNTIF(Issues!B2:B212,Stats!B12)</f>
-        <v>5</v>
+        <f>COUNTIF(Issues!B2:B213,Stats!B12)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -4207,7 +4184,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>68</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(Issues!B2:B214,Stats!B13)</f>
@@ -4219,7 +4196,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(Issues!B2:B215,Stats!B14)</f>
@@ -4227,25 +4204,13 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="2">
-        <v>13</v>
-      </c>
-      <c r="B15" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" s="2">
-        <f>COUNTIF(Issues!B2:B216,Stats!B15)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="C16" s="3">
-        <f>SUM(C3:C15)</f>
-        <v>192</v>
+      <c r="A15" s="4"/>
+      <c r="B15" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" s="3">
+        <f>SUM(C3:C14)</f>
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>